<commit_message>
Auswertung Planck fast fertig
</commit_message>
<xml_diff>
--- a/45/Evaluation/Data/Datasheet.xlsx
+++ b/45/Evaluation/Data/Datasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Moritz/Documents/GitHub/C-Praktikum/45/Evaluation/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C287D90-1342-014E-90A1-8B5B5D8B2F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E81B1D6E-AD59-FD48-A71A-14B7EDAB3DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2260" yWindow="2340" windowWidth="27380" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -531,12 +531,17 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="16.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.1640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.1640625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="15" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="20" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="16.33203125" style="2" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Auswertung Boltzmann fast fertig, nur Fehlerr K fehlt
</commit_message>
<xml_diff>
--- a/45/Evaluation/Data/Datasheet.xlsx
+++ b/45/Evaluation/Data/Datasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Moritz/Documents/GitHub/C-Praktikum/45/Evaluation/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{157FC8BD-1C44-D444-8806-5CF6450B1D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550D06A8-60A8-FC4F-910F-725E28A99BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17180" yWindow="940" windowWidth="16880" windowHeight="19340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>I (T=120 C)</t>
-  </si>
-  <si>
-    <t>Error I (T=120C)</t>
   </si>
   <si>
     <t>Error U (T=120 C)</t>
@@ -136,6 +133,9 @@
   </si>
   <si>
     <t>U (578nm)</t>
+  </si>
+  <si>
+    <t>Error I (T=120 C)</t>
   </si>
 </sst>
 </file>
@@ -551,67 +551,67 @@
   <sheetData>
     <row r="1" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="S1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2181,7 +2181,8 @@
     <col min="7" max="8" width="15.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="11" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="15.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="12.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.1640625" style="4" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" style="4" customWidth="1"/>
     <col min="16" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
@@ -2220,10 +2221,10 @@
         <v>10</v>
       </c>
       <c r="N1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2278,7 +2279,7 @@
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="C3" s="5">
-        <f t="shared" ref="C2:C24" si="2">B3*0.0005+10*0.00015</f>
+        <f t="shared" ref="C3:C24" si="2">B3*0.0005+10*0.00015</f>
         <v>1.5001999999999997E-3</v>
       </c>
       <c r="D3" s="5">

</xml_diff>